<commit_message>
allow runner with subset
</commit_message>
<xml_diff>
--- a/output/data_reports/latam_availability.xlsx
+++ b/output/data_reports/latam_availability.xlsx
@@ -4762,16 +4762,16 @@
         <v>14</v>
       </c>
       <c r="D160">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E160">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F160" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G160" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H160" t="s">
         <v>15</v>
@@ -4791,16 +4791,16 @@
         <v>14</v>
       </c>
       <c r="D161">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E161">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F161" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G161" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H161" t="s">
         <v>15</v>
@@ -4820,16 +4820,16 @@
         <v>14</v>
       </c>
       <c r="D162">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E162">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F162" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G162" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H162" t="s">
         <v>15</v>
@@ -4849,16 +4849,16 @@
         <v>14</v>
       </c>
       <c r="D163">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E163">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F163" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G163" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H163" t="s">
         <v>15</v>
@@ -5528,7 +5528,7 @@
         <v>14</v>
       </c>
       <c r="H186" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I186" t="s">
         <v>15</v>
@@ -5557,7 +5557,7 @@
         <v>14</v>
       </c>
       <c r="H187" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I187" t="s">
         <v>15</v>
@@ -5586,7 +5586,7 @@
         <v>14</v>
       </c>
       <c r="H188" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I188" t="s">
         <v>15</v>
@@ -5615,7 +5615,7 @@
         <v>14</v>
       </c>
       <c r="H189" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I189" t="s">
         <v>15</v>
@@ -5644,7 +5644,7 @@
         <v>14</v>
       </c>
       <c r="H190" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I190" t="s">
         <v>15</v>
@@ -5673,7 +5673,7 @@
         <v>14</v>
       </c>
       <c r="H191" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I191" t="s">
         <v>15</v>

</xml_diff>